<commit_message>
maj interaction matrix S2 et metadata
</commit_message>
<xml_diff>
--- a/interaction_matrix2.xlsx
+++ b/interaction_matrix2.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\stage_Curtin_Mahidol_2026\bobtail_pilot\bobtail_interactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AF6CF1-4862-4121-B751-A3063706E620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3741FAF-93BB-4DE4-9587-586B3B064946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AFA17CC3-2052-423B-B608-7260E968CD56}"/>
+    <workbookView xWindow="2295" yWindow="930" windowWidth="15375" windowHeight="9585" xr2:uid="{AFA17CC3-2052-423B-B608-7260E968CD56}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="interaction_matrix2" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -472,8 +472,8 @@
         <v>10</v>
       </c>
       <c r="G2">
-        <f>2+3+5+2+4</f>
-        <v>16</v>
+        <f>3+3+5+2+4</f>
+        <v>17</v>
       </c>
       <c r="H2">
         <f>2+1+3+1+2</f>
@@ -533,8 +533,8 @@
         <v>5</v>
       </c>
       <c r="G4">
-        <f>2+5+2+2+1</f>
-        <v>12</v>
+        <f>4+5+2+2+1</f>
+        <v>14</v>
       </c>
       <c r="H4">
         <f>2+1+1+3+5</f>
@@ -603,13 +603,13 @@
         <v>4</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>10</v>
       </c>
       <c r="D7">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E7">
         <v>9</v>

</xml_diff>

<commit_message>
split metadata between the 2 sessions + minor change to interaction matrix
</commit_message>
<xml_diff>
--- a/interaction_matrix2.xlsx
+++ b/interaction_matrix2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Desktop\stage_Curtin_Mahidol_2026\bobtail_pilot\bobtail_interactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3741FAF-93BB-4DE4-9587-586B3B064946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A3A109B-0852-44DB-B74E-0FB8097B9D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="930" windowWidth="15375" windowHeight="9585" xr2:uid="{AFA17CC3-2052-423B-B608-7260E968CD56}"/>
+    <workbookView xWindow="2340" yWindow="1335" windowWidth="15375" windowHeight="9585" xr2:uid="{AFA17CC3-2052-423B-B608-7260E968CD56}"/>
   </bookViews>
   <sheets>
     <sheet name="interaction_matrix2" sheetId="1" r:id="rId1"/>
@@ -440,8 +440,8 @@
         <v>3</v>
       </c>
       <c r="G1">
-        <f>1+2+1</f>
-        <v>4</v>
+        <f>1+2+3</f>
+        <v>6</v>
       </c>
       <c r="H1">
         <f>2+1+2+1+1</f>
@@ -533,8 +533,8 @@
         <v>5</v>
       </c>
       <c r="G4">
-        <f>4+5+2+2+1</f>
-        <v>14</v>
+        <f>4+5+2+2+2</f>
+        <v>15</v>
       </c>
       <c r="H4">
         <f>2+1+1+3+5</f>
@@ -600,7 +600,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>17</v>
@@ -609,7 +609,7 @@
         <v>10</v>
       </c>
       <c r="D7">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E7">
         <v>9</v>

</xml_diff>